<commit_message>
Add category classification sheets to Brita analysis
Adds two sheets to brita_analisis_DWI.xlsx:
- Resumen por categoria: the load split into 7 product categories with
  units, cost and share of spend.
- Clasificacion Savvy: per-UPC verdict, flagging consumables (filters)
  versus hardware (pitchers, dispensers, faucet systems, bottles) and
  marking the long tail of UPCs with 10 or fewer units.

Key figures: filters are 65% of cost (5,054 units across 12 UPCs);
hardware is 35% (1,999 units across 32 UPCs). 18 of the 44 UPCs carry
95.5% of the cost; the remaining 26 UPCs are 4.5%.

Also records that the seller priced every line at a flat 40% of MSRP
(Each) or 41% (Case), with no per-SKU differentiation.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQcJaksWjFxZHGRPHR6iFQ
</commit_message>
<xml_diff>
--- a/brita_analisis_DWI.xlsx
+++ b/brita_analisis_DWI.xlsx
@@ -12,6 +12,8 @@
     <sheet name="Detalle 73 lineas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Alertas datos" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Para buscar en eBay" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Resumen por categoria" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Clasificacion Savvy" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -733,8 +735,6 @@
       <c r="J3" t="n">
         <v>8.050000000000001</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -773,8 +773,6 @@
       <c r="J4" t="n">
         <v>7.22</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -909,8 +907,6 @@
       <c r="J7" t="n">
         <v>4.27</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -949,8 +945,6 @@
       <c r="J8" t="n">
         <v>2.11</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -989,8 +983,6 @@
       <c r="J9" t="n">
         <v>1.93</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1029,8 +1021,6 @@
       <c r="J10" t="n">
         <v>1.81</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1069,8 +1059,6 @@
       <c r="J11" t="n">
         <v>1.76</v>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1109,8 +1097,6 @@
       <c r="J12" t="n">
         <v>1.57</v>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1149,8 +1135,6 @@
       <c r="J13" t="n">
         <v>1.56</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1189,8 +1173,6 @@
       <c r="J14" t="n">
         <v>1.52</v>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1229,8 +1211,6 @@
       <c r="J15" t="n">
         <v>1.48</v>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1269,8 +1249,6 @@
       <c r="J16" t="n">
         <v>1.34</v>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1309,8 +1287,6 @@
       <c r="J17" t="n">
         <v>1.07</v>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1349,8 +1325,6 @@
       <c r="J18" t="n">
         <v>0.97</v>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1389,8 +1363,6 @@
       <c r="J19" t="n">
         <v>0.77</v>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1429,8 +1401,6 @@
       <c r="J20" t="n">
         <v>0.68</v>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1469,8 +1439,6 @@
       <c r="J21" t="n">
         <v>0.49</v>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1509,8 +1477,6 @@
       <c r="J22" t="n">
         <v>0.49</v>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1549,8 +1515,6 @@
       <c r="J23" t="n">
         <v>0.46</v>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1589,8 +1553,6 @@
       <c r="J24" t="n">
         <v>0.32</v>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1629,8 +1591,6 @@
       <c r="J25" t="n">
         <v>0.27</v>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1669,8 +1629,6 @@
       <c r="J26" t="n">
         <v>0.22</v>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1709,8 +1667,6 @@
       <c r="J27" t="n">
         <v>0.21</v>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1749,8 +1705,6 @@
       <c r="J28" t="n">
         <v>0.18</v>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1789,8 +1743,6 @@
       <c r="J29" t="n">
         <v>0.15</v>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1829,8 +1781,6 @@
       <c r="J30" t="n">
         <v>0.12</v>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1869,8 +1819,6 @@
       <c r="J31" t="n">
         <v>0.1</v>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1909,8 +1857,6 @@
       <c r="J32" t="n">
         <v>0.08</v>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1949,8 +1895,6 @@
       <c r="J33" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1989,8 +1933,6 @@
       <c r="J34" t="n">
         <v>0.05</v>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2029,8 +1971,6 @@
       <c r="J35" t="n">
         <v>0.04</v>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2069,8 +2009,6 @@
       <c r="J36" t="n">
         <v>0.04</v>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2109,8 +2047,6 @@
       <c r="J37" t="n">
         <v>0.03</v>
       </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2149,8 +2085,6 @@
       <c r="J38" t="n">
         <v>0.03</v>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2189,8 +2123,6 @@
       <c r="J39" t="n">
         <v>0.03</v>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2229,8 +2161,6 @@
       <c r="J40" t="n">
         <v>0.02</v>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2269,8 +2199,6 @@
       <c r="J41" t="n">
         <v>0.02</v>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2309,8 +2237,6 @@
       <c r="J42" t="n">
         <v>0.02</v>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2349,8 +2275,6 @@
       <c r="J43" t="n">
         <v>0.02</v>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2389,8 +2313,6 @@
       <c r="J44" t="n">
         <v>0.02</v>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2429,8 +2351,6 @@
       <c r="J45" t="n">
         <v>0.02</v>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2623,7 +2543,6 @@
           <t>0060258355017</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTERS 12/1CT</t>
@@ -2675,7 +2594,6 @@
           <t>0060258352146</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>BRITA BASE FAUCET FILTRATION SYSTEM WHITE 4/1CT</t>
@@ -2727,7 +2645,6 @@
           <t>0060258355017</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTERS 12/1CT</t>
@@ -2779,7 +2696,6 @@
           <t>0060258355031</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>BRITA PITCHER FILTERS 24/3CT SHIPPER</t>
@@ -2831,7 +2747,6 @@
           <t>0060258360899</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>BRITA SOHO PITCHER WHITE 2/1CT</t>
@@ -2883,7 +2798,6 @@
           <t>0060258360936</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>BRITA SOHO PITCHER COLOR1 2/1CT</t>
@@ -2935,7 +2849,6 @@
           <t>0060258363098</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>BRITA ON TAP REPLACEMENT FILTERS WHITE 6/1CT 1 TRAY</t>
@@ -2987,7 +2900,6 @@
           <t>0060258363104</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>BRITA ON TAP REPLACEMENT FILTERS CHROME 6/1CT 1 TRAY</t>
@@ -3039,7 +2951,6 @@
           <t>0060258364170</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTER 2/6CT</t>
@@ -3091,7 +3002,6 @@
           <t>0060258364590</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>BRITA ON TAP FILTRATION SYSTEM WHITE/WHITE W/EXTRA FILTER 4/1CT</t>
@@ -3143,7 +3053,6 @@
           <t>0060258365252</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>BRITA PREMIUM FILTERING BOTTLE HARD SIDED BLUSH 36OZ 6/1CT</t>
@@ -3195,7 +3104,6 @@
           <t>0060258508031</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>Brita Hub Filter 6/1ct SIOC</t>
@@ -3247,7 +3155,6 @@
           <t>0060258508031</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>BRITA HUB FILTER 6/1CT SIOC</t>
@@ -3299,7 +3206,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTER 10/10CT VALUE PALLET</t>
@@ -3351,7 +3257,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTER 10/10CT VALUE PALLET</t>
@@ -3403,7 +3308,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTER 10/10CT VALUE PALLET</t>
@@ -3567,7 +3471,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTER 10/10CT VALUE PALLET</t>
@@ -3619,7 +3522,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTER 10/10CT VALUE PALLET</t>
@@ -3671,7 +3573,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTER 10/10CT VALUE PALLET</t>
@@ -3723,7 +3624,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTER 10/10CT VALUE PALLET</t>
@@ -3775,7 +3675,6 @@
           <t>0060258509670</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>Brita Champlain Pitcher Bright White 100/1ct Value Pallet</t>
@@ -3827,7 +3726,6 @@
           <t>0060258355031</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>Brita Pitcher Filters 24/3ct Shipper</t>
@@ -3879,7 +3777,6 @@
           <t>0060258360899</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>Brita SOHO Pitcher White 2/1ct</t>
@@ -3931,7 +3828,6 @@
           <t>0060258362435</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>Brita Elite 12/1ct Sidekick Display</t>
@@ -3983,7 +3879,6 @@
           <t>0060258362619</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
           <t>Brita UltraMax Dispenser Jet Black with Elite Filter 2/1ct PK05</t>
@@ -4035,7 +3930,6 @@
           <t>0060258363128</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>Brita On Tap Replacement Filters Chrome 4/2ct 1 Tray</t>
@@ -4087,7 +3981,6 @@
           <t>0060258363159</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>BRITA ADVANCED PITCHER FILTER 8/8CT</t>
@@ -4139,7 +4032,6 @@
           <t>0060258364552</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
           <t>Brita SOHO Pitcher White w/Elite Filter 2/1ct</t>
@@ -4191,7 +4083,6 @@
           <t>0060258364606</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>Brita On Tap Filtration System Chrome/Chrome w/Extra Filter 4/1ct</t>
@@ -4243,7 +4134,6 @@
           <t>0060258364668</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>Brita Premium Filtering Bottle Hard Sided Orchid 36oz 6/1ct</t>
@@ -4295,7 +4185,6 @@
           <t>0060258365245</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>Brita Premium Filtering Bottle Hard Sided Sea Glass 36oz 6/1ct</t>
@@ -4347,7 +4236,6 @@
           <t>0060258506884</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
           <t>Brita Tahoe Pitcher w/ Elite+ Filter Bright White 2/1ct</t>
@@ -4399,7 +4287,6 @@
           <t>0060258509847</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>Brita Denali Pitcher Stone Blue 2/1ct</t>
@@ -4451,7 +4338,6 @@
           <t>0060258509854</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>Brita Tahoe Pitcher Stone Blue 2/1ct</t>
@@ -5175,7 +5061,6 @@
           <t>0060258509670</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
           <t>Brita Champlain Pitcher Bright White 100/1ct Value Pallet</t>
@@ -5227,7 +5112,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
           <t>Brita Advanced Pitcher Filter 10/10ct Value Pallet PK07</t>
@@ -5279,7 +5163,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
           <t>Brita Advanced Pitcher Filter 10/10ct Value Pallet PK07</t>
@@ -5331,7 +5214,6 @@
           <t>0060258355031</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
           <t>Brita Pitcher Filters 24/3ct Shipper</t>
@@ -5383,7 +5265,6 @@
           <t>0060258364545</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
           <t>Brita Bottle Replacement Filters Hard Sided 8/6ct</t>
@@ -5435,7 +5316,6 @@
           <t>0060258364552</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr">
         <is>
           <t>Brita SOHO Pitcher White w/Elite Filter 2/1ct</t>
@@ -5487,7 +5367,6 @@
           <t>0060258364606</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
           <t>Brita On Tap Filtration System Chrome/Chrome w/Extra Filter 4/1ct</t>
@@ -5539,7 +5418,6 @@
           <t>0060258356182</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
           <t>Brita On Tap Filtration System Chrome/Chrome 4/1ct</t>
@@ -5591,7 +5469,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
           <t>Brita Advanced Pitcher Filter 10/10ct Value Pallet PK07</t>
@@ -5643,7 +5520,6 @@
           <t>0060258360899</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr">
         <is>
           <t>Brita SOHO Pitcher White 2/1ct</t>
@@ -5695,7 +5571,6 @@
           <t>0060258364606</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
           <t>Brita On Tap Filtration System Chrome/Chrome w/Extra Filter 4/1ct</t>
@@ -5803,7 +5678,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
           <t>Brita Advanced Pitcher Filter 10/10ct Value Pallet PK07</t>
@@ -5855,7 +5729,6 @@
           <t>0060258509670</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
           <t>Brita Champlain Pitcher Bright White 100/1ct Value Pallet</t>
@@ -5907,7 +5780,6 @@
           <t>0060258507263</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
           <t>Brita Wave Pitcher White 2ct Elite 54/1ct Value Pallet PK01</t>
@@ -5959,7 +5831,6 @@
           <t>0060258507263</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
           <t>Brita Wave Pitcher White 2ct Elite 54/1ct Value Pallet PK01</t>
@@ -6011,7 +5882,6 @@
           <t>0060258507928</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
           <t>Brita UltraMax Dispenser Mazarine Blue 2/1ct</t>
@@ -6175,7 +6045,6 @@
           <t>0060258356182</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
           <t>Brita On Tap Filtration System Chrome/Chrome 4/1ct</t>
@@ -6227,7 +6096,6 @@
           <t>0060258509670</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
           <t>Brita Champlain Pitcher Bright White 100/1ct Value Pallet</t>
@@ -6391,7 +6259,6 @@
           <t>0060258359916</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr">
         <is>
           <t>Brita Advanced Pitcher Filter 10/10ct Value Pallet PK07</t>
@@ -7429,4 +7296,2152 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Cat</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>UPCs</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Unidades</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>% costo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Veredicto</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>4889</v>
+      </c>
+      <c r="D2" t="n">
+        <v>44185.15144</v>
+      </c>
+      <c r="E2" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SI - nucleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1198</v>
+      </c>
+      <c r="D3" t="n">
+        <v>16198.0989</v>
+      </c>
+      <c r="E3" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sistema grifo</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>623</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6339.34384</v>
+      </c>
+      <c r="E4" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" t="n">
+        <v>94</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1174.415</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>NO - cola larga</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Filtro botella</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>136</v>
+      </c>
+      <c r="D6" t="n">
+        <v>745.8240000000001</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>84</v>
+      </c>
+      <c r="D7" t="n">
+        <v>597.839959</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>MIXTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Filtro grifo</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="n">
+        <v>29</v>
+      </c>
+      <c r="D8" t="n">
+        <v>205.028</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SI - poco volumen</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="29" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>UPC</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cat</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Unidades_retail</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>MSRP_und</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Costo_und</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Costo_total</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>% del costo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Veredicto</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>060258359916</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BRITA ADVANCED PITCHER FILTER 10/10CT VALUE PALLET</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2082</v>
+      </c>
+      <c r="F2" t="n">
+        <v>39.27</v>
+      </c>
+      <c r="G2" t="n">
+        <v>15.71</v>
+      </c>
+      <c r="H2" t="n">
+        <v>32707.2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>SI - nucleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>060258355017</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BRITA ADVANCED PITCHER FILTERS 12/1CT</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5589.168000000001</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>SI - nucleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>060258362435</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Brita Elite 12/1ct Sidekick Display</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>432</v>
+      </c>
+      <c r="F4" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2967.552</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>SI - nucleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>060258508031</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Brita Hub Filter 6/1ct SIOC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>156</v>
+      </c>
+      <c r="F5" t="n">
+        <v>19.54</v>
+      </c>
+      <c r="G5" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1219.53144</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>SI - nucleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>060258364545</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Brita Bottle Replacement Filters Hard Sided 8/6ct</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Filtro botella</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>136</v>
+      </c>
+      <c r="F6" t="n">
+        <v>13.71</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="H6" t="n">
+        <v>745.8240000000001</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>060258355031</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BRITA PITCHER FILTERS 24/3CT SHIPPER</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>109</v>
+      </c>
+      <c r="F7" t="n">
+        <v>15.47</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="H7" t="n">
+        <v>674.564</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>SI - nucleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>060258363159</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BRITA ADVANCED PITCHER FILTER 8/8CT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>40</v>
+      </c>
+      <c r="F8" t="n">
+        <v>33.29</v>
+      </c>
+      <c r="G8" t="n">
+        <v>13.32</v>
+      </c>
+      <c r="H8" t="n">
+        <v>532.64</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>SI - nucleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>060258362442</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Brita Elite Pitcher Filters 8/2ct FM01</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>40</v>
+      </c>
+      <c r="F9" t="n">
+        <v>28.88</v>
+      </c>
+      <c r="G9" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="H9" t="n">
+        <v>473.632</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>SI - nucleo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>060258363128</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Brita On Tap Replacement Filters Chrome 4/2ct 1 Tray</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Filtro grifo</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F10" t="n">
+        <v>23.41</v>
+      </c>
+      <c r="G10" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>103.004</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>SI - poco volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>060258363104</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BRITA ON TAP REPLACEMENT FILTERS CHROME 6/1CT 1 TRAY</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Filtro grifo</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" t="n">
+        <v>14.17</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="H11" t="n">
+        <v>68.01600000000001</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>SI - poco volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>060258363098</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BRITA ON TAP REPLACEMENT FILTERS WHITE 6/1CT 1 TRAY</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Filtro grifo</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" t="n">
+        <v>14.17</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="H12" t="n">
+        <v>34.008</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>060258364170</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BRITA ADVANCED PITCHER FILTER 2/6CT</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>26.08</v>
+      </c>
+      <c r="G13" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="H13" t="n">
+        <v>20.864</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>060258356182</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Brita On Tap Filtration System Chrome/Chrome 4/1ct</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Sistema grifo</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>524</v>
+      </c>
+      <c r="F14" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="G14" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="H14" t="n">
+        <v>5013.632000000001</v>
+      </c>
+      <c r="I14" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>060258364552</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Brita SOHO Pitcher White w/Elite Filter 2/1ct</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>140</v>
+      </c>
+      <c r="F15" t="n">
+        <v>78.56999999999999</v>
+      </c>
+      <c r="G15" t="n">
+        <v>32.17</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4503.755200000001</v>
+      </c>
+      <c r="I15" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>060258509670</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Brita Champlain Pitcher Bright White 100/1ct Value Pallet</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>283</v>
+      </c>
+      <c r="F16" t="n">
+        <v>29.46</v>
+      </c>
+      <c r="G16" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3334.872</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>060258507263</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Brita Wave Pitcher White 2ct Elite 54/1ct Value Pallet PK01</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>98</v>
+      </c>
+      <c r="F17" t="n">
+        <v>37.31</v>
+      </c>
+      <c r="G17" t="n">
+        <v>14.92</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1462.552</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>060258365153</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BRITA PACIFICA PITCHER WHITE W/LONGLAST FILTER 2/1CT</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>96</v>
+      </c>
+      <c r="F18" t="n">
+        <v>34.11</v>
+      </c>
+      <c r="G18" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1342.5696</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>060258364606</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Brita On Tap Filtration System Chrome/Chrome w/Extra Filter 4/1ct</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sistema grifo</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>93</v>
+      </c>
+      <c r="F19" t="n">
+        <v>33.86</v>
+      </c>
+      <c r="G19" t="n">
+        <v>13.54</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1259.592</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>060258509878</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Brita Plus Everyday Pitcher - Clear 10 Cup</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>93</v>
+      </c>
+      <c r="F20" t="n">
+        <v>28.67</v>
+      </c>
+      <c r="G20" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1093.1871</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>060258507492</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BRITA ULTRAMAX DISPENSER GRAY 1/1CT SIOC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>88</v>
+      </c>
+      <c r="F21" t="n">
+        <v>30.06</v>
+      </c>
+      <c r="G21" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1084.5648</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>NO - cola larga</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>060258506846</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BRITA TAHOE PITCHER BRIGHT WHITE 2/1CT</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>96</v>
+      </c>
+      <c r="F22" t="n">
+        <v>26.77</v>
+      </c>
+      <c r="G22" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1053.6672</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>060258507010</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Brita Everyday Pitcher W/Smart Light Indicator Teal 1/1ct</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>96</v>
+      </c>
+      <c r="F23" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="G23" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1030.4448</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>060258507447</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Brita Metro Pitcher White SIOC 1/1ct</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>144</v>
+      </c>
+      <c r="F24" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="G24" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="H24" t="n">
+        <v>929.88</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>060258360899</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BRITA SOHO PITCHER WHITE 2/1CT</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>52</v>
+      </c>
+      <c r="F25" t="n">
+        <v>16.18</v>
+      </c>
+      <c r="G25" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="H25" t="n">
+        <v>341.7968</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>060258365252</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BRITA PREMIUM FILTERING BOTTLE HARD SIDED BLUSH 36OZ 6/1CT</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>48</v>
+      </c>
+      <c r="F26" t="n">
+        <v>17.63</v>
+      </c>
+      <c r="G26" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="H26" t="n">
+        <v>338.496</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>MIXTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>060258506884</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Brita Tahoe Pitcher w/ Elite+ Filter Bright White 2/1ct</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>24</v>
+      </c>
+      <c r="F27" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="G27" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="H27" t="n">
+        <v>321.792</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>060258506891</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Brita Tahoe Pitcher w/ Elite Filter Black 2/1ct</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>16</v>
+      </c>
+      <c r="F28" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="G28" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="H28" t="n">
+        <v>219.8912</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>060258509885</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Brita Plus Metro Pitcher - Stone Blue 6 Cup</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>28</v>
+      </c>
+      <c r="F29" t="n">
+        <v>16.62</v>
+      </c>
+      <c r="G29" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="H29" t="n">
+        <v>190.7976</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>060258508956</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Brita Everyday Pitcher w/ Smart Light Indicator w/ Refillable Filter SIOC 1ct</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>182.34</v>
+      </c>
+      <c r="G30" t="n">
+        <v>74.76000000000001</v>
+      </c>
+      <c r="H30" t="n">
+        <v>149.5188</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>060258360936</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BRITA SOHO PITCHER COLOR1 2/1CT</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>23</v>
+      </c>
+      <c r="F31" t="n">
+        <v>15.78</v>
+      </c>
+      <c r="G31" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="H31" t="n">
+        <v>148.601</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>MIXTO - depende del volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>060258365245</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Brita Premium Filtering Bottle Hard Sided Sea Glass 36oz 6/1ct</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>18</v>
+      </c>
+      <c r="F32" t="n">
+        <v>17.43</v>
+      </c>
+      <c r="G32" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="H32" t="n">
+        <v>125.496</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>MIXTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>060258364668</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Brita Premium Filtering Bottle Hard Sided Orchid 36oz 6/1ct</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>12</v>
+      </c>
+      <c r="F33" t="n">
+        <v>17.43</v>
+      </c>
+      <c r="G33" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="H33" t="n">
+        <v>83.664</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>MIXTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>060258364590</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BRITA ON TAP FILTRATION SYSTEM WHITE/WHITE W/EXTRA FILTER 4/1CT</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Sistema grifo</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" t="n">
+        <v>34.16</v>
+      </c>
+      <c r="G34" t="n">
+        <v>13.66</v>
+      </c>
+      <c r="H34" t="n">
+        <v>54.65584</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>060258364521</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Brita Premium Filtering Bottle Stainless Rose 20oz 6/1ct</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>6</v>
+      </c>
+      <c r="F35" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G35" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="H35" t="n">
+        <v>50.183959</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>060258362619</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Brita UltraMax Dispenser Jet Black with Elite Filter 2/1ct PK05</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" t="n">
+        <v>36.26</v>
+      </c>
+      <c r="G36" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="H36" t="n">
+        <v>29.008</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>060258507041</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Brita Everyday Pitcher W/Smart Light Indicator w/LongLast+ Filter Mazarine Blue 1/1ct</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="G37" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="H37" t="n">
+        <v>27.4864</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>060258507508</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Brita UltraMax Dispenser Black 1/1ct SIOC</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>57.76</v>
+      </c>
+      <c r="G38" t="n">
+        <v>23.68</v>
+      </c>
+      <c r="H38" t="n">
+        <v>23.6816</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>060258509854</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Brita Tahoe Pitcher Stone Blue 2/1ct</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="G39" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="H39" t="n">
+        <v>20.944</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>060258507027</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Brita Everyday Pitcher w/ Smart Light Indicator w/ Elite+ Filter BrightBright White 1/1ct</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="G40" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="H40" t="n">
+        <v>13.7432</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>060258509724</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Brita Ultramax Dispenser Brita Plus White SIOC 1/1ct</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="n">
+        <v>31.23</v>
+      </c>
+      <c r="G41" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H41" t="n">
+        <v>12.8043</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>060258509410</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Brita Ultramax Dispenser Translucent Jet Black w/ Brita Plus 1/1ct SIOC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>31.23</v>
+      </c>
+      <c r="G42" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H42" t="n">
+        <v>12.8043</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>060258509847</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Brita Denali Pitcher Stone Blue 2/1ct</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="G43" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H43" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>060258507928</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Brita UltraMax Dispenser Mazarine Blue 2/1ct</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>28.88</v>
+      </c>
+      <c r="G44" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="H44" t="n">
+        <v>11.552</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>060258352146</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>BRITA BASE FAUCET FILTRATION SYSTEM WHITE 4/1CT</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Sistema grifo</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" t="n">
+        <v>14.33</v>
+      </c>
+      <c r="G45" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="H45" t="n">
+        <v>11.464</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>NO - cola larga (&lt;=10 und)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add pallet lot breakdown to Brita analysis
Groups the 31 pallet-channel UPCs into four sellable lots and prices
each at 50% of retail, the default the Savvy Scanner applies.

New sheets in brita_analisis_DWI.xlsx:
- Lotes pallet: the four lots with units, cost, MSRP and margin.
- Pallet detalle: every pallet-channel UPC with its lot assignment.

Lots: A - loose 1ct filters (2,028 units, $5,589); B - volume pitchers
(7 SKUs, 792 units, $7,975); C - bottles (4 SKUs, 84 units, $598);
D - mixed long tail (19 SKUs, 179 units, $2,059).

At 50% of retail the whole pallet channel sells for $20,086 against
$16,221 of cost, a 24% return that is nearly identical across all four
lots because the seller priced every line at a flat 40% of MSRP.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQcJaksWjFxZHGRPHR6iFQ
</commit_message>
<xml_diff>
--- a/brita_analisis_DWI.xlsx
+++ b/brita_analisis_DWI.xlsx
@@ -17,6 +17,8 @@
     <sheet name="Canal MARKETPLACE" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Canal PALLET" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Notas y escenarios" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Lotes pallet" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Pallet detalle" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -681,7 +683,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -725,7 +726,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -736,6 +736,1322 @@
         <is>
           <t>Precios reales de eBay. Faltan por bloqueo de red; estos numeros son estimados.</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lote</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SKUs</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unidades</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>MSRP</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Venta @50% retail</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Utilidad</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ROI %</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Costo/und</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A - Filtros sueltos 1ct</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5589.168000000001</v>
+      </c>
+      <c r="E2" t="n">
+        <v>13972.92</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6986.46</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1397.29</v>
+      </c>
+      <c r="H2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2.76</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B - Pitchers de volumen</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3" t="n">
+        <v>792</v>
+      </c>
+      <c r="D3" t="n">
+        <v>7974.6455</v>
+      </c>
+      <c r="E3" t="n">
+        <v>19661.41</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9830.700000000001</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1856.05</v>
+      </c>
+      <c r="H3" t="n">
+        <v>23</v>
+      </c>
+      <c r="I3" t="n">
+        <v>10.07</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C - Botellas</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>84</v>
+      </c>
+      <c r="D4" t="n">
+        <v>597.839959</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1491.54</v>
+      </c>
+      <c r="F4" t="n">
+        <v>745.77</v>
+      </c>
+      <c r="G4" t="n">
+        <v>147.93</v>
+      </c>
+      <c r="H4" t="n">
+        <v>25</v>
+      </c>
+      <c r="I4" t="n">
+        <v>7.12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>19</v>
+      </c>
+      <c r="C5" t="n">
+        <v>179</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2059.21144</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5045.29</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2522.64</v>
+      </c>
+      <c r="G5" t="n">
+        <v>463.43</v>
+      </c>
+      <c r="H5" t="n">
+        <v>23</v>
+      </c>
+      <c r="I5" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lote</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>UPC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Cat</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unidades_retail</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MSRP_und</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Costo_und</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Costo_total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A - Filtros sueltos 1ct</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>060258355017</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>BRITA ADVANCED PITCHER FILTERS 12/1CT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5589.168000000001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B - Pitchers de volumen</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>060258509670</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Brita Champlain Pitcher Bright White 100/1ct Value Pallet</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>283</v>
+      </c>
+      <c r="F3" t="n">
+        <v>29.46</v>
+      </c>
+      <c r="G3" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3334.872</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B - Pitchers de volumen</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>060258509878</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Brita Plus Everyday Pitcher - Clear 10 Cup</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>93</v>
+      </c>
+      <c r="F4" t="n">
+        <v>28.67</v>
+      </c>
+      <c r="G4" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1093.1871</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B - Pitchers de volumen</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>060258506846</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BRITA TAHOE PITCHER BRIGHT WHITE 2/1CT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>96</v>
+      </c>
+      <c r="F5" t="n">
+        <v>26.77</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1053.6672</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B - Pitchers de volumen</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>060258507010</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Brita Everyday Pitcher W/Smart Light Indicator Teal 1/1ct</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>96</v>
+      </c>
+      <c r="F6" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1030.4448</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B - Pitchers de volumen</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>060258507447</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Brita Metro Pitcher White SIOC 1/1ct</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>144</v>
+      </c>
+      <c r="F7" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="H7" t="n">
+        <v>929.88</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B - Pitchers de volumen</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>060258360899</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BRITA SOHO PITCHER WHITE 2/1CT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>52</v>
+      </c>
+      <c r="F8" t="n">
+        <v>16.18</v>
+      </c>
+      <c r="G8" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="H8" t="n">
+        <v>341.7968</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B - Pitchers de volumen</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>060258509885</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Brita Plus Metro Pitcher - Stone Blue 6 Cup</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>28</v>
+      </c>
+      <c r="F9" t="n">
+        <v>16.62</v>
+      </c>
+      <c r="G9" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="H9" t="n">
+        <v>190.7976</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>C - Botellas</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>060258365252</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BRITA PREMIUM FILTERING BOTTLE HARD SIDED BLUSH 36OZ 6/1CT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>48</v>
+      </c>
+      <c r="F10" t="n">
+        <v>17.63</v>
+      </c>
+      <c r="G10" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="H10" t="n">
+        <v>338.496</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C - Botellas</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>060258365245</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Brita Premium Filtering Bottle Hard Sided Sea Glass 36oz 6/1ct</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>18</v>
+      </c>
+      <c r="F11" t="n">
+        <v>17.43</v>
+      </c>
+      <c r="G11" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="H11" t="n">
+        <v>125.496</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C - Botellas</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>060258364668</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Brita Premium Filtering Bottle Hard Sided Orchid 36oz 6/1ct</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F12" t="n">
+        <v>17.43</v>
+      </c>
+      <c r="G12" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="H12" t="n">
+        <v>83.664</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C - Botellas</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>060258364521</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Brita Premium Filtering Bottle Stainless Rose 20oz 6/1ct</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Botella</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="H13" t="n">
+        <v>50.183959</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>060258507492</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BRITA ULTRAMAX DISPENSER GRAY 1/1CT SIOC</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>88</v>
+      </c>
+      <c r="F14" t="n">
+        <v>30.06</v>
+      </c>
+      <c r="G14" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1084.5648</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>060258506891</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Brita Tahoe Pitcher w/ Elite Filter Black 2/1ct</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>16</v>
+      </c>
+      <c r="F15" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="G15" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="H15" t="n">
+        <v>219.8912</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>060258508956</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Brita Everyday Pitcher w/ Smart Light Indicator w/ Refillable Filter SIOC 1ct</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>182.34</v>
+      </c>
+      <c r="G16" t="n">
+        <v>74.76000000000001</v>
+      </c>
+      <c r="H16" t="n">
+        <v>149.5188</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>060258360936</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BRITA SOHO PITCHER COLOR1 2/1CT</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>23</v>
+      </c>
+      <c r="F17" t="n">
+        <v>15.78</v>
+      </c>
+      <c r="G17" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="H17" t="n">
+        <v>148.601</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>060258363128</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Brita On Tap Replacement Filters Chrome 4/2ct 1 Tray</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Filtro grifo</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>11</v>
+      </c>
+      <c r="F18" t="n">
+        <v>23.41</v>
+      </c>
+      <c r="G18" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="H18" t="n">
+        <v>103.004</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>060258363104</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BRITA ON TAP REPLACEMENT FILTERS CHROME 6/1CT 1 TRAY</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Filtro grifo</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" t="n">
+        <v>14.17</v>
+      </c>
+      <c r="G19" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="H19" t="n">
+        <v>68.01600000000001</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>060258364590</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BRITA ON TAP FILTRATION SYSTEM WHITE/WHITE W/EXTRA FILTER 4/1CT</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Sistema grifo</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" t="n">
+        <v>34.16</v>
+      </c>
+      <c r="G20" t="n">
+        <v>13.66</v>
+      </c>
+      <c r="H20" t="n">
+        <v>54.65584</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>060258363098</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BRITA ON TAP REPLACEMENT FILTERS WHITE 6/1CT 1 TRAY</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Filtro grifo</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>6</v>
+      </c>
+      <c r="F21" t="n">
+        <v>14.17</v>
+      </c>
+      <c r="G21" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="H21" t="n">
+        <v>34.008</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>060258362619</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Brita UltraMax Dispenser Jet Black with Elite Filter 2/1ct PK05</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>36.26</v>
+      </c>
+      <c r="G22" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="H22" t="n">
+        <v>29.008</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>060258507041</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Brita Everyday Pitcher W/Smart Light Indicator w/LongLast+ Filter Mazarine Blue 1/1ct</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="G23" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="H23" t="n">
+        <v>27.4864</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>060258507508</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Brita UltraMax Dispenser Black 1/1ct SIOC</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>57.76</v>
+      </c>
+      <c r="G24" t="n">
+        <v>23.68</v>
+      </c>
+      <c r="H24" t="n">
+        <v>23.6816</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>060258509854</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Brita Tahoe Pitcher Stone Blue 2/1ct</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="G25" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="H25" t="n">
+        <v>20.944</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>060258364170</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BRITA ADVANCED PITCHER FILTER 2/6CT</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Filtro pitcher</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>26.08</v>
+      </c>
+      <c r="G26" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="H26" t="n">
+        <v>20.864</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>060258507027</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Brita Everyday Pitcher w/ Smart Light Indicator w/ Elite+ Filter BrightBright White 1/1ct</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="G27" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="H27" t="n">
+        <v>13.7432</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>060258509724</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Brita Ultramax Dispenser Brita Plus White SIOC 1/1ct</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>31.23</v>
+      </c>
+      <c r="G28" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H28" t="n">
+        <v>12.8043</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>060258509410</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Brita Ultramax Dispenser Translucent Jet Black w/ Brita Plus 1/1ct SIOC</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>31.23</v>
+      </c>
+      <c r="G29" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H29" t="n">
+        <v>12.8043</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>060258509847</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Brita Denali Pitcher Stone Blue 2/1ct</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Pitcher</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="G30" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H30" t="n">
+        <v>12.6</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>060258507928</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Brita UltraMax Dispenser Mazarine Blue 2/1ct</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Dispenser</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>28.88</v>
+      </c>
+      <c r="G31" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="H31" t="n">
+        <v>11.552</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>D - Mixto / cola larga</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>060258352146</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BRITA BASE FAUCET FILTRATION SYSTEM WHITE 4/1CT</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Sistema grifo</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>14.33</v>
+      </c>
+      <c r="G32" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="H32" t="n">
+        <v>11.464</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark shipping rates as confirmed rather than estimated
Octavio reviewed the per-category shipping figures and confirmed they
match what he actually pays, so the sheet no longer asks for real rates
to replace them and RESULTADO FINAL no longer lists shipping as an open
estimate. No figures changed: the load still returns $19,971 on
$69,446 of cost (29%).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQcJaksWjFxZHGRPHR6iFQ
</commit_message>
<xml_diff>
--- a/brita_analisis_DWI.xlsx
+++ b/brita_analisis_DWI.xlsx
@@ -78,13 +78,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -709,7 +710,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ESTIMADO. Ver pestana "Tarifas envio" y reemplazar con tus tarifas reales.</t>
+          <t>CONFIRMADAS por Octavio (29-sep-2026). Ver pestana "Tarifas envio".</t>
         </is>
       </c>
     </row>
@@ -6655,13 +6656,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="47" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="53" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6675,14 +6675,9 @@
           <t>Nota</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Mi estimado $</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>TU TARIFA REAL $ &lt;- LLENAR</t>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Tarifa usada $ (CONFIRMADA por Octavio 29-sep-2026)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Label shipping rates as approximate and add a sensitivity table
Corrects the previous commit, which recorded the shipping figures as
confirmed. Octavio validated them by eye as roughly right, not as exact
rates, and the workbook now says so.

Adds a Sensibilidad envio sheet showing what the approximation is worth:
3,970 units go through the marketplace channel, so every $1 of error in
per-unit shipping moves the result by $3,970. At the figures used the
load returns $19,978 (29%); $1 cheaper returns 34%, $1 dearer 23%.

No headline figures changed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQcJaksWjFxZHGRPHR6iFQ
</commit_message>
<xml_diff>
--- a/brita_analisis_DWI.xlsx
+++ b/brita_analisis_DWI.xlsx
@@ -22,6 +22,7 @@
     <sheet name="Pallet detalle" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Precios eBay" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Tarifas envio" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Sensibilidad envio" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -710,7 +711,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CONFIRMADAS por Octavio (29-sep-2026). Ver pestana "Tarifas envio".</t>
+          <t>APROXIMADO. Validado de vista por Octavio (29-sep-2026). Cada $1 de diferencia mueve $3,970 - ver pestana "Sensibilidad envio".</t>
         </is>
       </c>
     </row>
@@ -6661,7 +6662,7 @@
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="47" customWidth="1" min="2" max="2"/>
-    <col width="53" customWidth="1" min="3" max="3"/>
+    <col width="61" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6675,9 +6676,9 @@
           <t>Nota</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>Tarifa usada $ (CONFIRMADA por Octavio 29-sep-2026)</t>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tarifa usada $ (APROXIMADA - validada de vista por Octavio)</t>
         </is>
       </c>
     </row>
@@ -6829,6 +6830,169 @@
       </c>
       <c r="C13" t="n">
         <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="70" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cada $1 de diferencia en el envio = $3,970 en el resultado final (3,970 unidades van por marketplace).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Si el envio real resulta</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Neto total</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>ROI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>-$3 por unidad</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>$31,888</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>46%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>-$2 por unidad</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>$27,918</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>-$1 por unidad</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>$23,948</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>34%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>COMO SE ESTIMO</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>$19,978</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>29%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>+$1 por unidad</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>$16,008</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>23%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>+$2 por unidad</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>$12,038</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>17%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>+$3 por unidad</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>$8,068</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>